<commit_message>
Search long_note und cv
</commit_message>
<xml_diff>
--- a/data/db/miniCRM/candidates_examples.xlsx
+++ b/data/db/miniCRM/candidates_examples.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bcwgruppe-my.sharepoint.com/personal/528337_fom-net_de/Documents/Git/KI_unterstuetztes_BMS_v1/KI-unterstuetztes-BMS/data/db/miniCRM/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="35" documentId="11_08B2CF4D9AFB9C608E3EE0254893406FF894F0B0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8FD9AF6D-01D9-4261-95B6-2CB33AD80BF6}"/>
+  <xr:revisionPtr revIDLastSave="47" documentId="11_08B2CF4D9AFB9C608E3EE0254893406FF894F0B0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A79BF9F7-CA18-4F9E-8E91-6A3A82DF300E}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="212" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18474,7 +18474,7 @@
       <c r="C2" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="5" t="s">
         <v>21</v>
       </c>
       <c r="E2" s="2" t="s">
@@ -18526,7 +18526,7 @@
       <c r="C3" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="5" t="s">
         <v>32</v>
       </c>
       <c r="E3" s="2" t="s">
@@ -18582,7 +18582,7 @@
       <c r="C4" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="5" t="s">
         <v>41</v>
       </c>
       <c r="E4" s="2" t="s">
@@ -18634,7 +18634,7 @@
       <c r="C5" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" s="5" t="s">
         <v>48</v>
       </c>
       <c r="E5" s="2" t="s">
@@ -18688,7 +18688,7 @@
       <c r="C6" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="D6" s="5" t="s">
         <v>52</v>
       </c>
       <c r="E6" s="2" t="s">
@@ -18740,7 +18740,7 @@
       <c r="C7" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="D7" s="5" t="s">
         <v>59</v>
       </c>
       <c r="E7" s="2" t="s">
@@ -18964,7 +18964,7 @@
       <c r="C12" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="D12" s="5" t="s">
         <v>79</v>
       </c>
       <c r="E12" s="2" t="s">
@@ -19248,7 +19248,7 @@
       <c r="C18" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="D18" s="2" t="s">
+      <c r="D18" s="5" t="s">
         <v>103</v>
       </c>
       <c r="E18" s="2" t="s">
@@ -19460,7 +19460,7 @@
         <v>66</v>
       </c>
       <c r="C22" s="2"/>
-      <c r="D22" s="2" t="s">
+      <c r="D22" s="5" t="s">
         <v>125</v>
       </c>
       <c r="E22" s="2" t="s">
@@ -19730,7 +19730,7 @@
       <c r="C29" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="D29" s="2" t="s">
+      <c r="D29" s="5" t="s">
         <v>142</v>
       </c>
       <c r="E29" s="2" t="s">
@@ -19806,7 +19806,7 @@
         <v>66</v>
       </c>
       <c r="C31" s="2"/>
-      <c r="D31" s="2" t="s">
+      <c r="D31" s="5" t="s">
         <v>149</v>
       </c>
       <c r="E31" s="2" t="s">
@@ -20113,7 +20113,7 @@
       <c r="B39" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="C39" s="2" t="s">
+      <c r="C39" s="5" t="s">
         <v>162</v>
       </c>
       <c r="D39" s="2"/>

</xml_diff>